<commit_message>
đảm bảo đúng thứ tự và tên file xuất ra
</commit_message>
<xml_diff>
--- a/kma_mm/kma_be/src/exports/excel/danh_gia_diem_qua_trinh.xlsx
+++ b/kma_mm/kma_be/src/exports/excel/danh_gia_diem_qua_trinh.xlsx
@@ -181,19 +181,28 @@
     <t>1</t>
   </si>
   <si>
+    <t>test0101</t>
+  </si>
+  <si>
+    <t>Nguyễn Văn Hòa</t>
+  </si>
+  <si>
+    <t>test01</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>test0102</t>
   </si>
   <si>
     <t>Lê Thị Bình</t>
   </si>
   <si>
-    <t>test01</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>2</t>
+    <t>3</t>
   </si>
   <si>
     <t>test0103</t>
@@ -202,22 +211,13 @@
     <t>Cao Huy Cường</t>
   </si>
   <si>
-    <t>3</t>
+    <t>4</t>
   </si>
   <si>
     <t>test0104</t>
   </si>
   <si>
     <t>Phạm Minh Dũng</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>test0101</t>
-  </si>
-  <si>
-    <t>Nguyễn Văn Hòa</t>
   </si>
   <si>
     <t>5</t>
@@ -1007,10 +1007,10 @@
         <v>29</v>
       </c>
       <c r="I15" s="8">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J15" s="8">
-        <v>9</v>
+        <v>8.2</v>
       </c>
       <c r="K15" s="8" t="s">
         <v>30</v>
@@ -1041,10 +1041,10 @@
         <v>29</v>
       </c>
       <c r="I16" s="8">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J16" s="8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K16" s="8" t="s">
         <v>30</v>
@@ -1075,10 +1075,10 @@
         <v>29</v>
       </c>
       <c r="I17" s="8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J17" s="8">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="K17" s="8" t="s">
         <v>30</v>
@@ -1112,7 +1112,7 @@
         <v>7</v>
       </c>
       <c r="J18" s="8">
-        <v>8.2</v>
+        <v>6.5</v>
       </c>
       <c r="K18" s="8" t="s">
         <v>30</v>

</xml_diff>